<commit_message>
chore: update coa taxonomy and codes
</commit_message>
<xml_diff>
--- a/data/coa_code.xlsx
+++ b/data/coa_code.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="28800" windowHeight="12180" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="BUMDES" sheetId="3" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="223">
   <si>
     <t>code</t>
   </si>
@@ -206,199 +206,208 @@
     <t>kewajiban</t>
   </si>
   <si>
-    <t>kewajiban_jk_pendek</t>
+    <t>kewajiban_jangka_pendek</t>
   </si>
   <si>
     <t>2.1.03.01</t>
   </si>
   <si>
+    <t>Utang Bagi Hasil BUMDES</t>
+  </si>
+  <si>
+    <t>utang_bagi_hasil_bumdes</t>
+  </si>
+  <si>
+    <t>3.1.01.01</t>
+  </si>
+  <si>
+    <t>Penyertaan Modal Desa</t>
+  </si>
+  <si>
+    <t>ekuitas</t>
+  </si>
+  <si>
+    <t>modal_desa</t>
+  </si>
+  <si>
+    <t>3.1.02.01</t>
+  </si>
+  <si>
+    <t>Penyertaan Modal Masyarakat</t>
+  </si>
+  <si>
+    <t>modal_masyarakat</t>
+  </si>
+  <si>
+    <t>3.2.01.01</t>
+  </si>
+  <si>
+    <t>Bagi Hasil Penyertaan Modal Desa</t>
+  </si>
+  <si>
+    <t>bagi_hasil_desa</t>
+  </si>
+  <si>
+    <t>3.2.02.01</t>
+  </si>
+  <si>
+    <t>Bagi Hasil Penyertaan Modal Masyarakat</t>
+  </si>
+  <si>
+    <t>bagi_hasil_masyarakat</t>
+  </si>
+  <si>
+    <t>3.3.01.01</t>
+  </si>
+  <si>
+    <t>Saldo Laba</t>
+  </si>
+  <si>
+    <t>saldo_laba</t>
+  </si>
+  <si>
+    <t>3.3.01.02</t>
+  </si>
+  <si>
+    <t>Laba Dicadangkan</t>
+  </si>
+  <si>
+    <t>laba_dicadangkan</t>
+  </si>
+  <si>
+    <t>3.9.01.01</t>
+  </si>
+  <si>
+    <t>Ikhtisar Laba Rugi</t>
+  </si>
+  <si>
+    <t>ikhtisar_laba_rugi</t>
+  </si>
+  <si>
+    <t>4.1.01.01</t>
+  </si>
+  <si>
+    <t>Pendapatan Usaha</t>
+  </si>
+  <si>
+    <t>pendapatan</t>
+  </si>
+  <si>
+    <t>pendapatan_operasional</t>
+  </si>
+  <si>
+    <t>4.1.01.02</t>
+  </si>
+  <si>
+    <t>Pendapatan Bagi Hasil</t>
+  </si>
+  <si>
+    <t>4.2.01.01</t>
+  </si>
+  <si>
+    <t>Pendapatan Lain-lain</t>
+  </si>
+  <si>
+    <t>pendapatan_lain_lain</t>
+  </si>
+  <si>
+    <t>4.2.01.02</t>
+  </si>
+  <si>
+    <t>Bunga Bank</t>
+  </si>
+  <si>
+    <t>5.1.01.01</t>
+  </si>
+  <si>
+    <t>Harga Pokok Penjualan Barang Dagangan</t>
+  </si>
+  <si>
+    <t>hpp</t>
+  </si>
+  <si>
+    <t>hpp_barang_dagangan</t>
+  </si>
+  <si>
+    <t>5.2.01.01</t>
+  </si>
+  <si>
+    <t>Harga Pokok Penjualan Barang Jadi</t>
+  </si>
+  <si>
+    <t>hpp_barang_jadi</t>
+  </si>
+  <si>
+    <t>6.1.01.01</t>
+  </si>
+  <si>
+    <t>Beban Administrasi Umum</t>
+  </si>
+  <si>
+    <t>beban</t>
+  </si>
+  <si>
+    <t>beban_administrasi</t>
+  </si>
+  <si>
+    <t>6.1.99.01</t>
+  </si>
+  <si>
+    <t>Beban Administrasi Lainnya</t>
+  </si>
+  <si>
+    <t>6.2.01.01</t>
+  </si>
+  <si>
+    <t>Beban Operasional Umum</t>
+  </si>
+  <si>
+    <t>beban_operasional</t>
+  </si>
+  <si>
+    <t>6.2.99.01</t>
+  </si>
+  <si>
+    <t>Beban Operasional Lainnya</t>
+  </si>
+  <si>
+    <t>6.3.01.01</t>
+  </si>
+  <si>
+    <t>Admin Bank</t>
+  </si>
+  <si>
+    <t>beban_lain_lain</t>
+  </si>
+  <si>
+    <t>6.3.01.02</t>
+  </si>
+  <si>
+    <t>Pajak Bunga Bank</t>
+  </si>
+  <si>
+    <t>1.1.01.11</t>
+  </si>
+  <si>
+    <t>Kas/Bank - UU01</t>
+  </si>
+  <si>
+    <t>UU01</t>
+  </si>
+  <si>
+    <t>1.1.03.11</t>
+  </si>
+  <si>
+    <t>2.1.01.11</t>
+  </si>
+  <si>
+    <t>2.1.03.11</t>
+  </si>
+  <si>
     <t>Utang Bagi Hasil</t>
   </si>
   <si>
-    <t>3.1.01.01</t>
-  </si>
-  <si>
-    <t>Penyertaan Modal Desa</t>
-  </si>
-  <si>
-    <t>ekuitas</t>
-  </si>
-  <si>
-    <t>modal_desa</t>
-  </si>
-  <si>
-    <t>3.1.02.01</t>
-  </si>
-  <si>
-    <t>Penyertaan Modal Masyarakat</t>
-  </si>
-  <si>
-    <t>modal_masyarakat</t>
-  </si>
-  <si>
-    <t>3.2.01.01</t>
-  </si>
-  <si>
-    <t>Bagi Hasil Penyertaan Modal Desa</t>
-  </si>
-  <si>
-    <t>bagi_hasil_desa</t>
-  </si>
-  <si>
-    <t>3.2.02.01</t>
-  </si>
-  <si>
-    <t>Bagi Hasil Penyertaan Modal Masyarakat</t>
-  </si>
-  <si>
-    <t>bagi_hasil_masyarakat</t>
-  </si>
-  <si>
-    <t>3.3.01.01</t>
-  </si>
-  <si>
-    <t>Saldo Laba</t>
-  </si>
-  <si>
-    <t>saldo_laba</t>
-  </si>
-  <si>
-    <t>3.3.01.02</t>
-  </si>
-  <si>
-    <t>Laba Dicadangkan</t>
-  </si>
-  <si>
-    <t>laba_dicadangkan</t>
-  </si>
-  <si>
-    <t>3.9.01.01</t>
-  </si>
-  <si>
-    <t>Ikhtisar Laba Rugi</t>
-  </si>
-  <si>
-    <t>ikhtisar_laba_rugi</t>
-  </si>
-  <si>
-    <t>4.1.01.01</t>
-  </si>
-  <si>
-    <t>Pendapatan Usaha</t>
-  </si>
-  <si>
-    <t>pendapatan</t>
-  </si>
-  <si>
-    <t>pendapatan_operasional</t>
-  </si>
-  <si>
-    <t>4.1.01.02</t>
-  </si>
-  <si>
-    <t>Pendapatan Bagi Hasil</t>
-  </si>
-  <si>
-    <t>4.2.01.01</t>
-  </si>
-  <si>
-    <t>Pendapatan Lain-lain</t>
-  </si>
-  <si>
-    <t>pendapatan_lain_lain</t>
-  </si>
-  <si>
-    <t>4.2.01.02</t>
-  </si>
-  <si>
-    <t>Bunga Bank</t>
-  </si>
-  <si>
-    <t>5.1.01.01</t>
-  </si>
-  <si>
-    <t>Harga Pokok Penjualan Barang Dagangan</t>
-  </si>
-  <si>
-    <t>hpp</t>
-  </si>
-  <si>
-    <t>hpp_barang_dagangan</t>
-  </si>
-  <si>
-    <t>5.2.01.01</t>
-  </si>
-  <si>
-    <t>Harga Pokok Penjualan Barang Jadi</t>
-  </si>
-  <si>
-    <t>hpp_barang_jadi</t>
-  </si>
-  <si>
-    <t>6.1.01.01</t>
-  </si>
-  <si>
-    <t>Beban Administrasi Umum</t>
-  </si>
-  <si>
-    <t>beban</t>
-  </si>
-  <si>
-    <t>beban_administrasi</t>
-  </si>
-  <si>
-    <t>6.1.99.01</t>
-  </si>
-  <si>
-    <t>Beban Administrasi Lainnya</t>
-  </si>
-  <si>
-    <t>6.2.01.01</t>
-  </si>
-  <si>
-    <t>Beban Operasional Umum</t>
-  </si>
-  <si>
-    <t>beban_operasional</t>
-  </si>
-  <si>
-    <t>6.2.99.01</t>
-  </si>
-  <si>
-    <t>Beban Operasional Lainnya</t>
-  </si>
-  <si>
-    <t>6.3.01.01</t>
-  </si>
-  <si>
-    <t>Admin Bank</t>
-  </si>
-  <si>
-    <t>beban_lain_lain</t>
-  </si>
-  <si>
-    <t>6.3.01.02</t>
-  </si>
-  <si>
-    <t>Pajak Bunga Bank</t>
-  </si>
-  <si>
-    <t>1.1.01.11</t>
-  </si>
-  <si>
-    <t>Kas/Bank - UU01</t>
-  </si>
-  <si>
-    <t>UU01</t>
-  </si>
-  <si>
-    <t>1.1.03.11</t>
-  </si>
-  <si>
-    <t>2.1.01.11</t>
-  </si>
-  <si>
-    <t>2.1.03.11</t>
+    <t>utang_bagi_hasil_unit</t>
   </si>
   <si>
     <t>3.1.01.11</t>
@@ -1322,7 +1331,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1331,9 +1340,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -2309,7 +2315,7 @@
       <c r="C22" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E22" s="1" t="s">
@@ -2329,8 +2335,8 @@
       <c r="C23" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>57</v>
+      <c r="D23" s="1" t="s">
+        <v>60</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>40</v>
@@ -2341,16 +2347,16 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>40</v>
@@ -2361,16 +2367,16 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>40</v>
@@ -2381,16 +2387,16 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>10</v>
@@ -2401,16 +2407,16 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>10</v>
@@ -2421,16 +2427,16 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>40</v>
@@ -2441,16 +2447,16 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>40</v>
@@ -2461,16 +2467,16 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>40</v>
@@ -2481,16 +2487,16 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>40</v>
@@ -2501,16 +2507,16 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>40</v>
@@ -2521,16 +2527,16 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>40</v>
@@ -2541,16 +2547,16 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>90</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>40</v>
@@ -2561,16 +2567,16 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>10</v>
@@ -2581,16 +2587,16 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>10</v>
@@ -2601,16 +2607,16 @@
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>10</v>
@@ -2621,16 +2627,16 @@
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>10</v>
@@ -2641,16 +2647,16 @@
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>10</v>
@@ -2661,16 +2667,16 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D40" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>10</v>
@@ -2681,16 +2687,16 @@
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>10</v>
@@ -2701,16 +2707,16 @@
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>10</v>
@@ -2765,10 +2771,10 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>8</v>
@@ -2780,12 +2786,12 @@
         <v>10</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>17</v>
@@ -2800,12 +2806,12 @@
         <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>55</v>
@@ -2813,234 +2819,234 @@
       <c r="C4" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>59</v>
+        <v>123</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>57</v>
+      <c r="D5" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -3086,10 +3092,10 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>8</v>
@@ -3101,12 +3107,12 @@
         <v>10</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>17</v>
@@ -3121,12 +3127,12 @@
         <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>55</v>
@@ -3134,234 +3140,234 @@
       <c r="C4" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>59</v>
+        <v>123</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>57</v>
+      <c r="D5" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -3407,10 +3413,10 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>8</v>
@@ -3422,12 +3428,12 @@
         <v>10</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>17</v>
@@ -3442,12 +3448,12 @@
         <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>55</v>
@@ -3455,234 +3461,234 @@
       <c r="C4" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>59</v>
+        <v>123</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>57</v>
+      <c r="D5" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -3728,10 +3734,10 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>8</v>
@@ -3743,12 +3749,12 @@
         <v>10</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>17</v>
@@ -3763,12 +3769,12 @@
         <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>20</v>
@@ -3783,12 +3789,12 @@
         <v>10</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>55</v>
@@ -3796,234 +3802,234 @@
       <c r="C5" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>59</v>
+        <v>123</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>57</v>
+      <c r="D6" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -4069,10 +4075,10 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>8</v>
@@ -4084,12 +4090,12 @@
         <v>10</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>17</v>
@@ -4104,12 +4110,12 @@
         <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>22</v>
@@ -4124,12 +4130,12 @@
         <v>10</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>24</v>
@@ -4144,12 +4150,12 @@
         <v>10</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>55</v>
@@ -4157,254 +4163,254 @@
       <c r="C6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>59</v>
+        <v>123</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>57</v>
+      <c r="D7" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="1" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="1" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -4450,10 +4456,10 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>8</v>
@@ -4465,12 +4471,12 @@
         <v>10</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>17</v>
@@ -4485,12 +4491,12 @@
         <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>22</v>
@@ -4505,12 +4511,12 @@
         <v>10</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>24</v>
@@ -4525,12 +4531,12 @@
         <v>10</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>55</v>
@@ -4538,254 +4544,254 @@
       <c r="C6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>59</v>
+        <v>123</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>57</v>
+      <c r="D7" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="1" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="1" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>